<commit_message>
docs(testing): add evidence dossier 08, postman collection v2.1, real execution logs, and ISO 25010 reference model clarification
</commit_message>
<xml_diff>
--- a/docs/testing/EcoAlerta_Testware_Matriz_Casos_Ejecucion.xlsx
+++ b/docs/testing/EcoAlerta_Testware_Matriz_Casos_Ejecucion.xlsx
@@ -895,10 +895,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
     <col width="50" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -1061,12 +1061,24 @@
     <row r="14" ht="22" customHeight="1">
       <c r="A14" s="11" t="inlineStr">
         <is>
-          <t>Estándar de Calidad ISO 25010</t>
+          <t>Modelo de Calidad ISO 25010</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Evaluación formal de los 8 atributos de calidad: Adecuación funcional, Rendimiento, Compatibilidad, Usabilidad, Fiabilidad, Seguridad, Mantenibilidad y Portabilidad.</t>
+          <t>Adopción de ISO/IEC 25010 como marco de referencia metodológica y guía de buenas prácticas de calidad para mantener consistencia, sin pretensión de certificación externa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>Respaldo de Evidencias y Packs de Datos</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Cada caso de prueba cuenta con su Request, Response y Pack de Datos exacto registrado en el Dossier de Evidencias (08_DOSSIER_EVIDENCIAS_DE_PRUEBA.md) y en la colección oficial exportada de Postman.</t>
         </is>
       </c>
     </row>

</xml_diff>